<commit_message>
feat: enhance map and chart responsiveness with dynamic resizing and cleanup improvements
</commit_message>
<xml_diff>
--- a/Data/crop Water Req.xlsx
+++ b/Data/crop Water Req.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\All_Portals\Agriculture Portal V2.4\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90827F71-5A1B-449E-9558-95A7A1C33AF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{773A21D9-7F9D-4F31-B0E0-FB59AE1CF138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{798FFF3B-AE4F-45CB-8D33-0960C01D22D2}"/>
   </bookViews>
@@ -132,13 +132,13 @@
     <t>Rapeseed &amp; Mustard</t>
   </si>
   <si>
-    <t>Sesamum</t>
-  </si>
-  <si>
     <t>Cash crop</t>
   </si>
   <si>
     <t>Tobacco</t>
+  </si>
+  <si>
+    <t>Sesame</t>
   </si>
 </sst>
 </file>
@@ -306,6 +306,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -315,11 +320,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -829,7 +829,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -855,7 +855,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="21"/>
+      <c r="A3" s="24"/>
       <c r="B3" s="12" t="s">
         <v>14</v>
       </c>
@@ -879,7 +879,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+      <c r="A4" s="24" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="12" t="s">
@@ -905,7 +905,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="21"/>
+      <c r="A5" s="24"/>
       <c r="B5" s="12" t="s">
         <v>14</v>
       </c>
@@ -929,7 +929,7 @@
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+      <c r="A6" s="24" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="12" t="s">
@@ -955,7 +955,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="21"/>
+      <c r="A7" s="24"/>
       <c r="B7" s="12" t="s">
         <v>14</v>
       </c>
@@ -979,7 +979,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="24" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="12" t="s">
@@ -1005,7 +1005,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" s="21"/>
+      <c r="A9" s="24"/>
       <c r="B9" s="12" t="s">
         <v>14</v>
       </c>
@@ -1029,7 +1029,7 @@
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
+      <c r="A10" s="24" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="12" t="s">
@@ -1055,7 +1055,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="22"/>
+      <c r="A11" s="25"/>
       <c r="B11" s="13" t="s">
         <v>14</v>
       </c>
@@ -1281,14 +1281,14 @@
       <c r="G1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="J1" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="25" t="s">
-        <v>32</v>
+      <c r="K1" s="22" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1313,13 +1313,13 @@
       <c r="G2" s="19">
         <v>80.274250000000009</v>
       </c>
-      <c r="I2" s="23" t="s">
+      <c r="I2" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="J2" s="23" t="s">
+      <c r="J2" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="K2" s="23" t="s">
+      <c r="K2" s="20" t="s">
         <v>2</v>
       </c>
     </row>
@@ -1345,14 +1345,14 @@
       <c r="G3" s="19">
         <v>77.305850000000007</v>
       </c>
-      <c r="I3" s="23" t="s">
+      <c r="I3" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="J3" s="23" t="s">
+      <c r="J3" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="K3" s="23" t="s">
-        <v>33</v>
+      <c r="K3" s="20" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -1377,13 +1377,13 @@
       <c r="G4" s="19">
         <v>75.703449999999989</v>
       </c>
-      <c r="I4" s="23" t="s">
+      <c r="I4" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="J4" s="23" t="s">
+      <c r="J4" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="K4" s="23" t="s">
+      <c r="K4" s="20" t="s">
         <v>4</v>
       </c>
     </row>
@@ -1409,13 +1409,13 @@
       <c r="G5" s="19">
         <v>73.891050000000007</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="J5" s="23" t="s">
+      <c r="J5" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="K5" s="23"/>
+      <c r="K5" s="20"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="14">
@@ -1439,20 +1439,20 @@
       <c r="G6" s="19">
         <v>71.898650000000004</v>
       </c>
-      <c r="I6" s="23" t="s">
+      <c r="I6" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="J6" s="23" t="s">
+      <c r="J6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="23"/>
+      <c r="K6" s="20"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="I7" s="23"/>
-      <c r="J7" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="K7" s="23"/>
+      <c r="I7" s="20"/>
+      <c r="J7" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>